<commit_message>
fix(somtam): fix news syntax error, set food curation prompts, add 40 fresh products, and enhance review logging
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="630" yWindow="615" windowWidth="37095" windowHeight="17310" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4210,6 +4210,1006 @@
       <c r="G143" t="inlineStr">
         <is>
           <t>done 2026-07-29 20:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>37</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>น้ำมันถั่วเหลือง ตราองุ่น ขนาด1ลิตร แพ็ค3ขวด โปรโมชั่นสุดคุ้ม</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7AbMVrSjRr</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztg-mnmyv5cdh05e5b.webp</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>฿182.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>38</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>The Chocolate Factory บราวนี่แครกเกอร์ แผ่นกลม รสดาร์กช็อกโกแลต ขนาด 40 กรัม</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4VabKxlcAB</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztj-mlvtyt7kgburbc.webp</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>฿45.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>39</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Ensure Gold AdvancePro wheat เอนชัวร์ โกลด์ แอดวานซ์โปร รสข้าวสาลี ขนาด 800 กรัม(1กระป๋อง)</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1LdZZ95AAb</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztp-mngva2okzpjaca.webp</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>฿690.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>40</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>[พร้อมส่งในไทย]Marukyu Koyamaen Matcha มัทฉะมารุคิวโคยามะเอ็น สาหร่ายผู้ดี อูมามิ เกรดพิธีการญี่ปุ่น</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7pr3J5kKve</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7rasj-m91el64l52bt32.webp</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>฿1118.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>41</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>หมูสามชั้นแดดเดียวพรีเมี่ยม อบลมร้อน สะอาด ไร้ฝุ่น ไร้แมลง ไม่ใส่สารกันเสีย ทอดง่ายๆใน 5 นาที</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8pjaUvq9ci</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztq-mmfq4vxucrgla3.webp</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>฿189.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>42</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Country Sourdough Bread ขนมปังซาวโดว์โฮมเมด 100% | SOURDOUGH BREAD |</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/W4SZcVdkx</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7ra0h-mcpd1y74lysm7e.webp</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>฿182.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>43</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>[ยกลัง12ขวด]น้ำมันปาล์ม มรกต และ ทับทิม ขวด 1ลิตร x 12 ขวด น้ำมันพืช มรกต และ ทับทิม</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2BCgYgRq4z</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81zth-mmixuw8fz18i52.webp</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>฿893.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>44</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>มัทฉะ Kanbayashi Shunsho Usucha Aya no Mori อายะ โนะ โมริ 20g/40g Uji matcha【ส่งตรงจากญี่ปุ่น】</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1VwzlSdFG1</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztd-mj8j4x9o8jd27f.webp</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>฿1451.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>45</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Pre-order มาม่าJinmailang (จางหลิงเฮ่อ) แพค</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/AAEy5OGUk8</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztq-mni8oy7lbjer1f.webp</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>฿260.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>46</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>หอยจ๊อปูย่าเฮี๊ยะ (เกรดเนื้อหน้าอก)แถมฟรีน้ำจิ้มบ๊วย30ML</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8ATthiVwhF</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztn-mncpondjeg3nd1.webp</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>฿270.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>47</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>น้ำมันมรกต 1 ลิตร ยกลัง 12 ขวด สินค้าส่งตรงจากโรงงาน (1 คำสั่งซื้อ 1 ลัง) ต้องการมากกว่า 1 ให้แยกคำสั่งซื้อ</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5fmYj7nmUw</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7r98u-lnfj2bxeyxioc3.webp</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>฿822.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>48</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>พร้อมส่งในไทย Marukyu​ Koyamaen​ ผงมัทฉะ​ มารุคิวของแท้จากญี่ปุ่น​ Matcha​ มัทฉะยี่ห้อดังจากอูจิ</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6ff5uxshlo</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztq-mn5j25gwgmx2ed.webp</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>฿790.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>49</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>ปลาสลิดกรอบ ไร้ก้าง เต็มชิ้น กรอบอร่อย ไม่เหม็นหืน 🐟</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/40eKk4DAW1</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7qula-lhkogxzv71yba0.webp</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>฿150.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>50</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>หมูแดดเดียวพรีเมียม อบลมร้อน สะอาด ไร้ฝุ่น ไร้แมลง เนื้อนุ่ม ฉ่ำ ทอดง่าย</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6ff5uyAZwu</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztg-mm8rnpzzshs429.webp</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>฿149.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>51</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>ไร่พระจันทร์ เมล็ดเจีย chia seed เมล็ดเชีย ธัญพืช มีอย. คัดพิเศษ เกรดพรีเมี่ยม</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9030hGB78j</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7r98u-lyj1u7grm8w1bb.webp</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>฿165.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>52</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>น้ำมันมรกต ขนาด 1 ลิตร สำหรับทำอาหาร แพ็ค 3 ขวด | น้ำมันพืชทำอาหาร ผัด ทอด อเนกประสงค์ ใช้ได้ทุกเมนู</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/W4SZdljey</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztf-mm9msusd71fnbc.webp</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>฿280.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>53</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>เก๊กฮวยผงสำเร็จรูป HighlandHerb ขนาด 600 กรัม</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3B5DkXjty0</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7r98v-lp4vdgeuw77id2.webp</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>฿249.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>54</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>สลิดติดปาก ปลาสลิดแดดเดียว 5-6 ตัว/โล | ปลาสลิดไข่บางบ่อ ตัวโต สด สะอาด เนื้อแน่นหอมมัน</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4fu1XIoEEN</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztm-mgvmi6civ40e0a.webp</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>฿469.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>55</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>นมกล่อง (ยกลัง) นมยูเอชที นมไฮคิวสูตร3 1พลัส ซูเปอร์โกลด์ รสจืด180 มล (27 กล่อง) นม UHT HiQ Super Gold UHT</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3LOdwr0WRj</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7rasg-m7hrtewsksjj0d.webp</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>฿669.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>56</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>เบอร์ทอลี่น้ำมันมะกอกเอ็กตร้าเวอร์จิน ขนาด500ml.</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9030hGnxIf</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztq-mo16o8447m69aa.webp</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>฿560.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>57</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>พัดลมดูดอากาศติดฝ้า 8/10/12 นิ้ว แรงดูด 300CFM เงียบ ประหยัดไฟ พัดลมระบายอากาศห้องน้ำ รับประกัน 3 ปี</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1qaN0cYfkf</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zte-moysj4upxu6l2c.webp</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>฿479.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>58</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>MAILTANK เตาแก็ส IK03 เตาแก๊สหัวเดี่ยว เตาแก๊สพกพา ขนาดกะทัดรัด ไฟแรง ประหยัดแก๊ส พร้อมส่ง (ใช้กับหัวปรับแรงดันต่ำ)</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6AjMAaRBJL</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zth-mngmbtc89hc030.webp</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>฿229.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>59</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>พัดลมระบายอากาศ พัดลมระบายอากาศติดเพดาน 8 นิ้ว 12 นิ้ว ลมแรง เสียงเงียบ ประหยัดไฟ เหมาะกับห้องน้ำ ห้องครัว</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7KvJYjR8jG</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zte-mohmysxqeeq7a2.webp</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>฿479.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>60</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>COD✅ ชั้นแม่เหล็กติดข้างตู้เย็น ชั้นวางแม่เหล็ก ไม่ต้องเจาะผนัง แรงดูดสูง รับน้ำหนักดี เหมาะสำหรับห้องครัว ห้องนอน และห้องน้ำ ประหยัดพื้นที่</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3B5kb4pSRZ</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-821fp-mgndrxqlei2w9f.webp</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>฿44.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>61</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>ชั้นวางแก้วไม้ไผ่ ชั้นวางแก้วน้ำ ชั้นวางจาน ทนทานต่อแรงกด ขนาดเล็กและประหยัดพื้นที่ อุปกรณ์จัดเก็บในครัว</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/60PvyHnbm6</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-824gg-mpwi58v183d9f1.webp</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>฿45.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>62</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>ถังขยะ ถังขยะแบบพกพา ถังขยะในครัว ดีไซน์มินิมอล แรงแบริ่งที่แข็งแกร่ง ประหยัดพื้นที่ ความจุขนาดใหญ่ แบบฝาสวิง</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9zw4jdhFUM</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81zti-mhptex6zswsl5b.webp</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>฿48.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>63</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>แรงดันน้ําสูง 360° หัวก๊อกน้ําทองเหลือง สามโหมด ยืดหยุ่น ประหยัดน้ํา สําหรับอ่างล้างจาน ห้องครัว ในครัวเรือน</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/qhponP5B0</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-7r98o-lmfyed9dgiqs57.webp</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>฿276.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>64</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>เครื่องปั่นไข่อเนกประสงค์ อุปกรณ์ตีไข่และผสมไข่ ใช้งานสะดวก เขย่าได้แรง ประหยัดเวลา เหมาะทำอาหารในครัว</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/BS91ZaHZK</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-825zu-mjpf4xitpkaq0d.webp</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>฿89.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>65</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>ปืนจุดแก๊ส ปืนจุดแก๊สใส่ถ่าน AA แบบสปาร์ค จุดติดง่ายไฟแรงทนทานประหยัด</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4LHhzETDg9</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/a1b11015b4f86d5433baba12bd1f7e2b.webp</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>฿95.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>66</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>KUDSUN คีมแกะหอยแครง สแตนเลส ที่แกะหอยแครง อุปกรณ์แกะหอยทะเล ช่วยเปิดเปลือกหอยง่าย ประหยัดแรง ทำอาหาร ไม่เจ็บมือ</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7fY9xMPoJd</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-23020-kji2eakg95mv2a.webp</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>฿168.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>67</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>ที่หนีบไม้กวาดแบบดูดติดผนัง ถ้วยดูดแรงสูง ไม่ต้องเจาะ ใช้แขวนไม้กวาดและที่ถูพื้นได้ ประหยัดพื้นที่ในห้องน้ำและห้องครัว</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5VTfNNgVxy</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztq-mlrhd1qtruh06f.webp</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>฿197.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>68</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>【พร้อมส่ง】หัวต่อก๊อกน้ำ 360° หมุนได้ ABS 3โหมด แรงดันสูง ประหยัดน้ำ ติดตั้งง่าย สำหรับอ่างล้างจานและห้องครัว</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2qSuCU0hf9</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztq-mh06e1dr06j117.webp</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>฿17.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>69</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>（COD）ก๊อกน้ำอ่างล้างจาน 4in1 หัวก๊อกครัว 4โหมด แรงดันสูง หมุนได้รอบทิศ สำหรับซิงค์ล้างจาน ติดตั้งง่าย ประหยัดน้ำ ล้างผัก</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8V7Gwtmh0a</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-81ztg-migzx3z3d1j45e.webp</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>฿299.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>70</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>อุปกรณ์ครัว2โหมด360 หมุนได้ บับเบิ้ล แรงดันสูงก๊อกน้ํา ส่วนต่อขยาย ประหยัดน้ําห้องน้ําอุปกรณ์ครัวอุปกรณ์</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9fJEL2r3Cr</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-7ra3y-m52qjdz9ofmf74.webp</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>฿20.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>71</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>ที่คั้นน้ำส้ม ที่บีบมะนาว 2in1 คั้นมือ+หมุนได้ในอุปกรณ์เดียว ประหยัดแรง</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7KvJYl4x5Q</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/th-11134207-7rasd-m2m6flkttcwjb2.webp</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>฿109.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>72</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>หัวก๊อกน้ำเพิ่มแรงดัน แบบหมุนได้ 360 องศา เหมาะสำหรับใช้งานในห้องครัว หัวก๊อกน้ำฝักบัวประหยัดน้ำเพิ่มแรงดัน</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8Knqkb9fZa</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-7rdyw-lzaaluuiprqicf.webp</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>฿28.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>73</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>ก๊อกน้ำอ่างล้างจานแบบดึงออกสปริง360° อ่างล้างจานหมุนล้างจาน กะละมังผัก ก๊อกน้ำซิงค์ครัว หัวฉีดดึงได้ 2 หมุนรอบ 360° เพิ่มแรงดัน ประหยัดน้ำ ติดตั้งง่าย</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4qDyaAVJOz</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-820l4-mjfr089l0s8x21.webp</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>฿699.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>74</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>ก๊อกน้ําห้องครัวสากลกรองเครื่องกรองน้ําหัวฉีดในครัวเรือนแรงดันประหยัดน้ําสาดหลักฐานตาข่ายองค์ประกอบอะแดปเตอร์</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/70ITA9RSni</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/cn-11134207-7ras8-m1nv75ekn12s34.webp</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>฿64.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>75</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>ตะขอรางเลื่อนอเนกประสงค์ - 10 Gliding S-Hooks &amp; กาวเสริมแรง, ประหยัดพื้นที่ Organizer - สําหรับเครื่องมือครัว/หมวก Coats</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1qaN0etnJT</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-7rd5t-m7w0a1xbzp1t77.webp</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>฿33.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>76</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>【ปรับ 2 ระดับ/หมุน 360°】FM ก๊อกน้ำครัวแบบปรับแรงดันน้ำ หมุนได้รอบทิศทาง อุปกรณ์ประปาในบ้าน/ก๊อกน้ำปรับแรงดัน/ก๊อกน้ำห้องน้ำ/ก๊อกน้ำประหยัดน้ำ</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4qDyaArecr</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>https://down-tx-th.img.susercontent.com/sg-11134201-8262o-mlnangheu9z98f.webp</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>฿670.00</t>
         </is>
       </c>
     </row>

</xml_diff>